<commit_message>
Exported M1 Evo cell composition data
</commit_message>
<xml_diff>
--- a/__ReadMe.xlsx
+++ b/__ReadMe.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -5593,6 +5593,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
@@ -5601,15 +5610,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5856,26 +5856,26 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
edit typo and capitalization
</commit_message>
<xml_diff>
--- a/__ReadMe.xlsx
+++ b/__ReadMe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="149" documentId="13_ncr:1_{0FC7810F-34CA-C64C-B96F-ABDAC602D8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D7FDA6E-33B4-9E41-BE2B-0C7D2203B6D5}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="13_ncr:1_{0FC7810F-34CA-C64C-B96F-ABDAC602D8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0725EF1A-AA76-D147-92BB-751950291942}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="33080" windowHeight="21580" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33080" windowHeight="20280" activeTab="1" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -854,9 +854,6 @@
     <t xml:space="preserve">Ref last </t>
   </si>
   <si>
-    <t>if there are typos or shorthand speces names used, can update based on heading, note, text</t>
-  </si>
-  <si>
     <t>add a column to correct any errors in species designations (e.g., misidentified or combined different species of same genus)</t>
   </si>
   <si>
@@ -1008,6 +1005,9 @@
   </si>
   <si>
     <t>10.1159%2F000437413_Table1.tsv</t>
+  </si>
+  <si>
+    <t>if there are typos or shorthand species names used, can update based on heading, note, text</t>
   </si>
 </sst>
 </file>
@@ -1805,7 +1805,7 @@
         <v>21</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="Y1" s="6" t="s">
         <v>22</v>
@@ -1897,7 +1897,7 @@
         <v>10.1093%2Fjmammal%2Fgyz043_SupplementaryDataSD1.tsv</v>
       </c>
       <c r="O2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>42</v>
@@ -1986,7 +1986,7 @@
         <v>notfound</v>
       </c>
       <c r="O3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P3" t="s">
         <v>53</v>
@@ -2079,7 +2079,7 @@
         <v>notfound</v>
       </c>
       <c r="O4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P4" t="s">
         <v>53</v>
@@ -2170,7 +2170,7 @@
         <v>10.1007%2Fs004220000205_Figure3.tsv</v>
       </c>
       <c r="O5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="P5" t="s">
         <v>35</v>
@@ -2254,7 +2254,7 @@
         <v>10.1038%2Fs41467-020-14356-3_SupplementaryData3.tsv</v>
       </c>
       <c r="O6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="P6" t="s">
         <v>53</v>
@@ -2351,7 +2351,7 @@
         <v>10.1159%2F000452856_TableS1.tsv</v>
       </c>
       <c r="O7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="P7" t="s">
         <v>53</v>
@@ -2448,7 +2448,7 @@
         <v>10.1523%2FJNEUROSCI.2339-19.2020_Table1.tsv</v>
       </c>
       <c r="O8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="P8" t="s">
         <v>53</v>
@@ -2537,7 +2537,7 @@
         <v>10.1093%2Foso%2F9780198568742.003.0006_Table6.1.tsv</v>
       </c>
       <c r="O9" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P9" t="s">
         <v>35</v>
@@ -2629,7 +2629,7 @@
         <v>10.1159%2F000124401_TableI.tsv</v>
       </c>
       <c r="O10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="P10" t="s">
         <v>53</v>
@@ -2718,7 +2718,7 @@
         <v>notfound</v>
       </c>
       <c r="O11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P11" t="s">
         <v>35</v>
@@ -2794,7 +2794,7 @@
         <v>notfound</v>
       </c>
       <c r="O12" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P12" t="s">
         <v>35</v>
@@ -2863,7 +2863,7 @@
         <v>10.1159%2F000437413_Table1.tsv</v>
       </c>
       <c r="O13" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P13" t="s">
         <v>53</v>
@@ -2960,7 +2960,7 @@
         <v>10.1159%2F000437413_Table2.tsv</v>
       </c>
       <c r="O14" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P14" t="s">
         <v>53</v>
@@ -3054,7 +3054,7 @@
         <v>10.1159%2F000437413_Table3.tsv</v>
       </c>
       <c r="O15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P15" t="s">
         <v>53</v>
@@ -3148,7 +3148,7 @@
         <v>10.1159%2F000437413_Table4.tsv</v>
       </c>
       <c r="O16" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P16" t="s">
         <v>53</v>
@@ -3242,7 +3242,7 @@
         <v>10.1159%2F000437413_Table5.tsv</v>
       </c>
       <c r="O17" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P17" t="s">
         <v>53</v>
@@ -3336,7 +3336,7 @@
         <v>10.1002%2Fcne.24985_TABLE1.tsv</v>
       </c>
       <c r="O18" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="P18" t="s">
         <v>53</v>
@@ -3430,7 +3430,7 @@
         <v>10.1002%2Fcne.24985_TABLE2.tsv</v>
       </c>
       <c r="O19" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="P19" t="s">
         <v>53</v>
@@ -3526,7 +3526,7 @@
         <v>notfound</v>
       </c>
       <c r="O20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P20" t="s">
         <v>35</v>
@@ -3597,7 +3597,7 @@
         <v>notfound</v>
       </c>
       <c r="O21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P21" t="s">
         <v>35</v>
@@ -3668,7 +3668,7 @@
         <v>notfound</v>
       </c>
       <c r="O22" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P22" t="s">
         <v>35</v>
@@ -3739,7 +3739,7 @@
         <v>notfound</v>
       </c>
       <c r="O23" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P23" t="s">
         <v>35</v>
@@ -3810,7 +3810,7 @@
         <v>10.3389%2Ffnana.2017.00118_Table1.tsv</v>
       </c>
       <c r="O24" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P24" t="s">
         <v>53</v>
@@ -3907,13 +3907,13 @@
         <v>10.1038%2Fs41598-018-26062-8_Table1.tsv</v>
       </c>
       <c r="O25" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P25" t="s">
         <v>53</v>
       </c>
       <c r="Q25" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="R25" s="3" t="s">
         <v>55</v>
@@ -3929,10 +3929,10 @@
       </c>
       <c r="W25" s="8"/>
       <c r="X25" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="Y25" t="s">
         <v>265</v>
-      </c>
-      <c r="Y25" t="s">
-        <v>266</v>
       </c>
       <c r="Z25" t="s">
         <v>99</v>
@@ -3999,13 +3999,13 @@
         <v>10.1038%2Fs41598-018-26062-8_TableS1.tsv</v>
       </c>
       <c r="O26" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P26" t="s">
         <v>53</v>
       </c>
       <c r="Q26" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R26" s="3" t="s">
         <v>55</v>
@@ -4093,13 +4093,13 @@
         <v>10.1038%2Fs41598-018-26062-8_TableS5.tsv</v>
       </c>
       <c r="O27" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P27" t="s">
         <v>53</v>
       </c>
       <c r="Q27" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="R27" s="3" t="s">
         <v>55</v>
@@ -4187,7 +4187,7 @@
         <v>notfound</v>
       </c>
       <c r="O28" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P28" t="s">
         <v>35</v>
@@ -4271,7 +4271,7 @@
         <v>notfound</v>
       </c>
       <c r="O29" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P29" t="s">
         <v>35</v>
@@ -4355,7 +4355,7 @@
         <v>notfound</v>
       </c>
       <c r="O30" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P30" t="s">
         <v>35</v>
@@ -4435,7 +4435,7 @@
         <v>notfound</v>
       </c>
       <c r="O31" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P31" t="s">
         <v>35</v>
@@ -4510,7 +4510,7 @@
         <v>notfound</v>
       </c>
       <c r="O32" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P32" t="s">
         <v>35</v>
@@ -4580,7 +4580,7 @@
         <v>notfound</v>
       </c>
       <c r="O33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="P33" t="s">
         <v>35</v>
@@ -4644,7 +4644,7 @@
         <v>10.1126%2Fscience.aaa9101_TableS1.tsv</v>
       </c>
       <c r="O34" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="P34" s="3" t="s">
         <v>42</v>
@@ -4696,7 +4696,7 @@
         <v>10.3389%2Ffnana.2013.00035_Figure2TopLeft.tsv</v>
       </c>
       <c r="O35" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="P35" s="3" t="s">
         <v>42</v>
@@ -4745,7 +4745,7 @@
         <v>10.3389%2Ffnana.2013.00035_Table1-a.tsv</v>
       </c>
       <c r="O36" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="P36" s="3" t="s">
         <v>42</v>
@@ -4794,7 +4794,7 @@
         <v>10.3389%2Ffnana.2013.00035_Table1-b.tsv</v>
       </c>
       <c r="O37" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="P37" s="3" t="s">
         <v>42</v>
@@ -4843,7 +4843,7 @@
         <v>10.1016%2Fj.jhevol.2008.08.004_Table2.tsv</v>
       </c>
       <c r="O38" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P38" s="3" t="s">
         <v>42</v>
@@ -4895,7 +4895,7 @@
         <v>10.1016%2Fj.jhevol.2008.08.004_Table7.tsv</v>
       </c>
       <c r="O39" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P39" s="3" t="s">
         <v>42</v>
@@ -4947,7 +4947,7 @@
         <v>10.1016%2Fj.jhevol.2008.08.004_TableS1.tsv</v>
       </c>
       <c r="O40" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P40" s="3" t="s">
         <v>42</v>
@@ -4996,7 +4996,7 @@
         <v>10.1016%2Fj.jhevol.2008.08.004_TableS2.tsv</v>
       </c>
       <c r="O41" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P41" s="3" t="s">
         <v>42</v>
@@ -5051,7 +5051,7 @@
         <v>10.1016%2Fj.jhevol.2008.08.004_TableS3.tsv</v>
       </c>
       <c r="O42" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P42" s="3" t="s">
         <v>42</v>
@@ -5104,7 +5104,7 @@
         <v>notfound</v>
       </c>
       <c r="O43" s="17" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P43" s="20" t="s">
         <v>42</v>
@@ -5150,16 +5150,16 @@
         <v>10.1371%2Fjournal.pbio.1002000_TableS1.tsv</v>
       </c>
       <c r="O44" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="P44" s="3" t="s">
         <v>42</v>
       </c>
       <c r="X44" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA44" t="s">
         <v>270</v>
-      </c>
-      <c r="AA44" t="s">
-        <v>271</v>
       </c>
       <c r="AI44">
         <v>9</v>
@@ -5208,7 +5208,7 @@
         <v>10.1371%2Fjournal.pbio.1002000_TableS8.tsv</v>
       </c>
       <c r="O45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="P45" s="3" t="s">
         <v>42</v>
@@ -5217,7 +5217,7 @@
         <v>225</v>
       </c>
       <c r="AA45" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AI45">
         <v>6</v>
@@ -5277,7 +5277,7 @@
         <v>42</v>
       </c>
       <c r="AA46" s="17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AI46" s="17">
         <v>7</v>
@@ -5327,7 +5327,7 @@
         <v>10.1159%2F000323671_SupplementaryTable1.tsv</v>
       </c>
       <c r="O47" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="P47" s="23" t="s">
         <v>42</v>
@@ -5377,7 +5377,7 @@
         <v>10.1159%2F000323671_SupplementaryTable2.tsv</v>
       </c>
       <c r="O48" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="P48" s="23" t="s">
         <v>42</v>
@@ -5388,7 +5388,7 @@
     </row>
     <row r="49" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B49" s="22" t="str">
         <f t="shared" ref="B49:B52" si="68">C49 &amp; IF(D49&lt;&gt;"", "_" &amp; D49, "_") &amp; IF(E49&lt;&gt;"", "_" &amp; E49, "_") &amp; IF(F49&lt;&gt;"", "_" &amp; F49, "")</f>
@@ -5434,7 +5434,7 @@
         <v>notfound</v>
       </c>
       <c r="O49" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="V49" t="s">
         <v>78</v>
@@ -5442,7 +5442,7 @@
     </row>
     <row r="50" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B50" s="22" t="str">
         <f t="shared" si="68"/>
@@ -5485,18 +5485,18 @@
         <v>notfound</v>
       </c>
       <c r="O50" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="X50" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="AC50" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B51" s="22" t="str">
         <f t="shared" si="68"/>
@@ -5521,7 +5521,7 @@
       </c>
       <c r="H51" s="15"/>
       <c r="I51" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J51" s="23" t="str">
         <f t="shared" si="72"/>
@@ -5539,18 +5539,18 @@
         <v>notfound</v>
       </c>
       <c r="O51" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="X51" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="AC51" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B52" s="22" t="str">
         <f t="shared" si="68"/>
@@ -5593,30 +5593,30 @@
         <v>10.1159%2F000319019_Table1.tsv</v>
       </c>
       <c r="O52" s="15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="P52" t="s">
         <v>53</v>
       </c>
       <c r="Q52" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="X52" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Z52" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AC52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AE52" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B53" s="22" t="str">
         <f t="shared" ref="B53:B55" si="77">C53 &amp; IF(D53&lt;&gt;"", "_" &amp; D53, "_") &amp; IF(E53&lt;&gt;"", "_" &amp; E53, "_") &amp; IF(F53&lt;&gt;"", "_" &amp; F53, "")</f>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="H53" s="15"/>
       <c r="I53" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J53" s="23" t="str">
         <f t="shared" ref="J53:J54" si="82">TRIM(_xlfn.TEXTJOIN("_",FALSE,B53,(SUBSTITUTE(SUBSTITUTE(I53," ",""), "_", ""))))</f>
@@ -5655,34 +5655,34 @@
         <v>10.1159%2F000319019_SupplementaryTable1</v>
       </c>
       <c r="M53" s="15" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="N53" t="str" cm="1">
         <f t="array" ref="N53">IFERROR(INDEX([1]FileList!$A$1:$A$43, MATCH(K53, _xlfn.TEXTBEFORE([1]FileList!$A$1:$A$43, ".tsv"), 0)), "notfound")</f>
         <v>10.1159%2F000319019_SupplementaryTable1.tsv</v>
       </c>
       <c r="O53" s="15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="Q53" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="X53" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Z53" t="s">
+        <v>282</v>
+      </c>
+      <c r="AC53" t="s">
+        <v>285</v>
+      </c>
+      <c r="AE53" t="s">
         <v>283</v>
-      </c>
-      <c r="AC53" t="s">
-        <v>286</v>
-      </c>
-      <c r="AE53" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="54" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B54" s="22" t="str">
         <f t="shared" si="77"/>
@@ -5723,21 +5723,21 @@
         <v>notfound</v>
       </c>
       <c r="O54" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="X54" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Z54" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AC54" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B55" s="22" t="str">
         <f t="shared" si="77"/>
@@ -5778,10 +5778,10 @@
         <v>notfound</v>
       </c>
       <c r="O55" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="X55" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -5860,7 +5860,7 @@
         <v>242</v>
       </c>
       <c r="B7" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -5876,7 +5876,7 @@
         <v>245</v>
       </c>
       <c r="B9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -5983,12 +5983,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6235,20 +6237,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6273,18 +6282,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>